<commit_message>
chore(data): rebuild team KPIs and team master table
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RXNnq4YFBytwJMyKM4XiDM
</commit_message>
<xml_diff>
--- a/data/curated/team_master_table.xlsx
+++ b/data/curated/team_master_table.xlsx
@@ -11,12 +11,14 @@
     <sheet name="Master" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="BN Team Stats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dunkest Defense vs Position" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Team KPIs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Guide'!$A$1:$C$156</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master'!$A$1:$EW$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Guide'!$A$1:$C$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master'!$A$1:$FC$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BN Team Stats'!$A$1:$DX$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dunkest Defense vs Position'!$A$1:$AA$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Team KPIs'!$A$1:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C156"/>
+  <dimension ref="A1:C163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -3093,8 +3095,127 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>team_name</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Team name (Basketnews spelling); joins into the team master table</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>pace_factor</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>offense_all_possessions (Basketnews team stats, per-game pace) / the 20-team league average; 1.0 = league-average pace, &gt;1 = faster than average</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_drawn</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>offense_all_fouls_received (Basketnews team stats) per 40 minutes of team play; already a per-game average and a game is 40 regulation minutes, so under a fixed 40-minutes-per-game assumption (overtime not modeled, no per-game minutes data exists) this equals the raw per-game rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_committed</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>defense_all_fouls (Basketnews team stats, fouls the team itself commits) per 40 minutes of team play; same 40-minutes-per-game assumption as foul_rate_per40_drawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>funnel_ratio_guards</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>guards_fantasy_points (Dunkest defense vs position, conceded per game) / the 20-team league average for guards; 1.0 = league-average funnel to guards, &gt;1 = concedes more than average</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>funnel_ratio_forwards</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>forwards_fantasy_points (Dunkest defense vs position, conceded per game) / the 20-team league average for forwards</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>funnel_ratio_centers</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>centers_fantasy_points (Dunkest defense vs position, conceded per game) / the 20-team league average for centers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C156"/>
+  <autoFilter ref="A1:C163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3105,7 +3226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EW21"/>
+  <dimension ref="A1:FC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3261,6 +3382,12 @@
     <col width="27" customWidth="1" min="151" max="151"/>
     <col width="41" customWidth="1" min="152" max="152"/>
     <col width="32" customWidth="1" min="153" max="153"/>
+    <col width="20" customWidth="1" min="154" max="154"/>
+    <col width="23" customWidth="1" min="155" max="155"/>
+    <col width="27" customWidth="1" min="156" max="156"/>
+    <col width="21" customWidth="1" min="157" max="157"/>
+    <col width="23" customWidth="1" min="158" max="158"/>
+    <col width="22" customWidth="1" min="159" max="159"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4029,6 +4156,36 @@
           <t>dunkdvp_centers_fantasy_points</t>
         </is>
       </c>
+      <c r="EX1" s="1" t="inlineStr">
+        <is>
+          <t>pace_factor</t>
+        </is>
+      </c>
+      <c r="EY1" s="1" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_drawn</t>
+        </is>
+      </c>
+      <c r="EZ1" s="1" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_committed</t>
+        </is>
+      </c>
+      <c r="FA1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_guards</t>
+        </is>
+      </c>
+      <c r="FB1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_forwards</t>
+        </is>
+      </c>
+      <c r="FC1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_centers</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4494,6 +4651,24 @@
       <c r="EW2" t="n">
         <v>15.24</v>
       </c>
+      <c r="EX2" t="n">
+        <v>0.9756427604871448</v>
+      </c>
+      <c r="EY2" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="EZ2" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="FA2" t="n">
+        <v>0.9749853715623171</v>
+      </c>
+      <c r="FB2" t="n">
+        <v>1.07522518867159</v>
+      </c>
+      <c r="FC2" t="n">
+        <v>1.018886846063848</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4959,6 +5134,24 @@
       <c r="EW3" t="n">
         <v>15.11</v>
       </c>
+      <c r="EX3" t="n">
+        <v>1.012178619756428</v>
+      </c>
+      <c r="EY3" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="EZ3" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="FA3" t="n">
+        <v>0.9991222937390286</v>
+      </c>
+      <c r="FB3" t="n">
+        <v>0.9681084151586465</v>
+      </c>
+      <c r="FC3" t="n">
+        <v>1.010195554069865</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5424,6 +5617,24 @@
       <c r="EW4" t="n">
         <v>14.36</v>
       </c>
+      <c r="EX4" t="n">
+        <v>1.017591339648173</v>
+      </c>
+      <c r="EY4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="EZ4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="FA4" t="n">
+        <v>0.9208601521357519</v>
+      </c>
+      <c r="FB4" t="n">
+        <v>1.037896616083746</v>
+      </c>
+      <c r="FC4" t="n">
+        <v>0.9600534848738091</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5889,6 +6100,24 @@
       <c r="EW5" t="n">
         <v>14.45</v>
       </c>
+      <c r="EX5" t="n">
+        <v>0.9986468200270637</v>
+      </c>
+      <c r="EY5" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="EZ5" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="FA5" t="n">
+        <v>1.019602106495026</v>
+      </c>
+      <c r="FB5" t="n">
+        <v>0.9486326381562932</v>
+      </c>
+      <c r="FC5" t="n">
+        <v>0.9660705331773357</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6354,6 +6583,24 @@
       <c r="EW6" t="n">
         <v>14.81</v>
       </c>
+      <c r="EX6" t="n">
+        <v>0.9769959404600813</v>
+      </c>
+      <c r="EY6" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="EZ6" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="FA6" t="n">
+        <v>1.129315389116442</v>
+      </c>
+      <c r="FB6" t="n">
+        <v>0.9713543779923721</v>
+      </c>
+      <c r="FC6" t="n">
+        <v>0.9901387263914425</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6819,6 +7066,24 @@
       <c r="EW7" t="n">
         <v>15.22</v>
       </c>
+      <c r="EX7" t="n">
+        <v>0.9756427604871448</v>
+      </c>
+      <c r="EY7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="EZ7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="FA7" t="n">
+        <v>0.988150965476887</v>
+      </c>
+      <c r="FB7" t="n">
+        <v>0.9161730098190376</v>
+      </c>
+      <c r="FC7" t="n">
+        <v>1.01754972421862</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7284,6 +7549,24 @@
       <c r="EW8" t="n">
         <v>14.84</v>
       </c>
+      <c r="EX8" t="n">
+        <v>0.9810554803788905</v>
+      </c>
+      <c r="EY8" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="EZ8" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="FA8" t="n">
+        <v>0.9574312463428906</v>
+      </c>
+      <c r="FB8" t="n">
+        <v>1.008682950580216</v>
+      </c>
+      <c r="FC8" t="n">
+        <v>0.9921444091592847</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7749,6 +8032,24 @@
       <c r="EW9" t="n">
         <v>14.82</v>
       </c>
+      <c r="EX9" t="n">
+        <v>0.9742895805142086</v>
+      </c>
+      <c r="EY9" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="EZ9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="FA9" t="n">
+        <v>0.9062317144528964</v>
+      </c>
+      <c r="FB9" t="n">
+        <v>1.003002515621196</v>
+      </c>
+      <c r="FC9" t="n">
+        <v>0.9908072873140565</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8214,6 +8515,24 @@
       <c r="EW10" t="n">
         <v>12.63</v>
       </c>
+      <c r="EX10" t="n">
+        <v>1.001353179972936</v>
+      </c>
+      <c r="EY10" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="EZ10" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="FA10" t="n">
+        <v>0.9764482153306027</v>
+      </c>
+      <c r="FB10" t="n">
+        <v>0.9526900916984502</v>
+      </c>
+      <c r="FC10" t="n">
+        <v>0.8443924452615745</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8679,6 +8998,24 @@
       <c r="EW11" t="n">
         <v>15.65</v>
       </c>
+      <c r="EX11" t="n">
+        <v>1.032476319350474</v>
+      </c>
+      <c r="EY11" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="EZ11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="FA11" t="n">
+        <v>1.132241076653014</v>
+      </c>
+      <c r="FB11" t="n">
+        <v>1.113365251967865</v>
+      </c>
+      <c r="FC11" t="n">
+        <v>1.046297843891025</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9144,6 +9481,24 @@
       <c r="EW12" t="n">
         <v>17.7</v>
       </c>
+      <c r="EX12" t="n">
+        <v>0.9986468200270637</v>
+      </c>
+      <c r="EY12" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="EZ12" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="FA12" t="n">
+        <v>1.106641310708016</v>
+      </c>
+      <c r="FB12" t="n">
+        <v>0.9932646271200196</v>
+      </c>
+      <c r="FC12" t="n">
+        <v>1.18335283302691</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9609,6 +9964,24 @@
       <c r="EW13" t="n">
         <v>16.15</v>
       </c>
+      <c r="EX13" t="n">
+        <v>1.032476319350474</v>
+      </c>
+      <c r="EY13" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="EZ13" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="FA13" t="n">
+        <v>1.075190169689877</v>
+      </c>
+      <c r="FB13" t="n">
+        <v>1.124726121885905</v>
+      </c>
+      <c r="FC13" t="n">
+        <v>1.079725890021728</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10074,6 +10447,24 @@
       <c r="EW14" t="n">
         <v>12.31</v>
       </c>
+      <c r="EX14" t="n">
+        <v>0.9972936400541274</v>
+      </c>
+      <c r="EY14" t="n">
+        <v>23</v>
+      </c>
+      <c r="EZ14" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="FA14" t="n">
+        <v>0.9771796372147454</v>
+      </c>
+      <c r="FB14" t="n">
+        <v>0.8918282885660961</v>
+      </c>
+      <c r="FC14" t="n">
+        <v>0.8229984957379242</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10539,6 +10930,24 @@
       <c r="EW15" t="n">
         <v>12.1</v>
       </c>
+      <c r="EX15" t="n">
+        <v>0.9864682002706362</v>
+      </c>
+      <c r="EY15" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="EZ15" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="FA15" t="n">
+        <v>1.088355763604447</v>
+      </c>
+      <c r="FB15" t="n">
+        <v>0.9324028239876655</v>
+      </c>
+      <c r="FC15" t="n">
+        <v>0.8089587163630286</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11004,6 +11413,24 @@
       <c r="EW16" t="n">
         <v>19.07</v>
       </c>
+      <c r="EX16" t="n">
+        <v>1.056833558863329</v>
+      </c>
+      <c r="EY16" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="EZ16" t="n">
+        <v>23</v>
+      </c>
+      <c r="FA16" t="n">
+        <v>1.040813341135167</v>
+      </c>
+      <c r="FB16" t="n">
+        <v>1.097946928507669</v>
+      </c>
+      <c r="FC16" t="n">
+        <v>1.274945679425038</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11469,6 +11896,24 @@
       <c r="EW17" t="n">
         <v>18.21</v>
       </c>
+      <c r="EX17" t="n">
+        <v>0.9959404600811909</v>
+      </c>
+      <c r="EY17" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="EZ17" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="FA17" t="n">
+        <v>1.012287887653599</v>
+      </c>
+      <c r="FB17" t="n">
+        <v>1.001379534204333</v>
+      </c>
+      <c r="FC17" t="n">
+        <v>1.217449440080227</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11934,6 +12379,24 @@
       <c r="EW18" t="n">
         <v>11.4</v>
       </c>
+      <c r="EX18" t="n">
+        <v>0.9878213802435725</v>
+      </c>
+      <c r="EY18" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="EZ18" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="FA18" t="n">
+        <v>0.958894090111176</v>
+      </c>
+      <c r="FB18" t="n">
+        <v>0.9088695934431551</v>
+      </c>
+      <c r="FC18" t="n">
+        <v>0.7621594517800435</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12399,6 +12862,24 @@
       <c r="EW19" t="n">
         <v>13.9</v>
       </c>
+      <c r="EX19" t="n">
+        <v>1.029769959404601</v>
+      </c>
+      <c r="EY19" t="n">
+        <v>21</v>
+      </c>
+      <c r="EZ19" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="FA19" t="n">
+        <v>0.9603569338794616</v>
+      </c>
+      <c r="FB19" t="n">
+        <v>1.015174876247667</v>
+      </c>
+      <c r="FC19" t="n">
+        <v>0.9292996824335618</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12864,6 +13345,24 @@
       <c r="EW20" t="n">
         <v>16.03</v>
       </c>
+      <c r="EX20" t="n">
+        <v>0.9878213802435725</v>
+      </c>
+      <c r="EY20" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="EZ20" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="FA20" t="n">
+        <v>0.9566998244587478</v>
+      </c>
+      <c r="FB20" t="n">
+        <v>1.050880467418648</v>
+      </c>
+      <c r="FC20" t="n">
+        <v>1.071703158950359</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13329,9 +13828,27 @@
       <c r="EW21" t="n">
         <v>15.15</v>
       </c>
+      <c r="EX21" t="n">
+        <v>0.9810554803788905</v>
+      </c>
+      <c r="EY21" t="n">
+        <v>21</v>
+      </c>
+      <c r="EZ21" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="FA21" t="n">
+        <v>0.8191925102399062</v>
+      </c>
+      <c r="FB21" t="n">
+        <v>0.9883956828694312</v>
+      </c>
+      <c r="FC21" t="n">
+        <v>1.012869797760321</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:EW21"/>
+  <autoFilter ref="A1:FC21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23842,4 +24359,565 @@
   <autoFilter ref="A1:AA21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>team_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>pace_factor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_drawn</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>foul_rate_per40_committed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_guards</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_forwards</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_ratio_centers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Anadolu Efes Istanbul</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.9756427604871448</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9749853715623171</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.07522518867159</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.018886846063848</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AS Monaco</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.012178619756428</v>
+      </c>
+      <c r="C3" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9991222937390286</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9681084151586465</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.010195554069865</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Crvena Zvezda Meridianbet Belgrade</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.017591339648173</v>
+      </c>
+      <c r="C4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9208601521357519</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.037896616083746</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9600534848738091</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dubai Basketball</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.9986468200270637</v>
+      </c>
+      <c r="C5" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.019602106495026</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9486326381562932</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9660705331773357</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EA7 Emporio Armani Milan</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.9769959404600813</v>
+      </c>
+      <c r="C6" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.129315389116442</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.9713543779923721</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9901387263914425</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FC Barcelona</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.9756427604871448</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.988150965476887</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9161730098190376</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.01754972421862</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FC Bayern Munich</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.9810554803788905</v>
+      </c>
+      <c r="C8" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9574312463428906</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.008682950580216</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9921444091592847</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fenerbahce Beko Istanbul</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.9742895805142086</v>
+      </c>
+      <c r="C9" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9062317144528964</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.003002515621196</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.9908072873140565</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hapoel Shlomo Tel Aviv</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.001353179972936</v>
+      </c>
+      <c r="C10" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9764482153306027</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.9526900916984502</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.8443924452615745</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kosner Baskonia Vitoria-Gasteiz</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.032476319350474</v>
+      </c>
+      <c r="C11" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.132241076653014</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.113365251967865</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.046297843891025</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LDLC ASVEL Villeurbanne</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.9986468200270637</v>
+      </c>
+      <c r="C12" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.106641310708016</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9932646271200196</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.18335283302691</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Maccabi Playtika Tel Aviv</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1.032476319350474</v>
+      </c>
+      <c r="C13" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.075190169689877</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.124726121885905</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.079725890021728</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Olympiacos Piraeus</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.9972936400541274</v>
+      </c>
+      <c r="C14" t="n">
+        <v>23</v>
+      </c>
+      <c r="D14" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9771796372147454</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.8918282885660961</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.8229984957379242</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Panathinaikos AKTOR Athens</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.9864682002706362</v>
+      </c>
+      <c r="C15" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.088355763604447</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.9324028239876655</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.8089587163630286</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Paris Basketball</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.056833558863329</v>
+      </c>
+      <c r="C16" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>23</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.040813341135167</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.097946928507669</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.274945679425038</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Partizan Mozzart Bet Belgrade</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.9959404600811909</v>
+      </c>
+      <c r="C17" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.012287887653599</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.001379534204333</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.217449440080227</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.9878213802435725</v>
+      </c>
+      <c r="C18" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.958894090111176</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.9088695934431551</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.7621594517800435</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Valencia Basket</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.029769959404601</v>
+      </c>
+      <c r="C19" t="n">
+        <v>21</v>
+      </c>
+      <c r="D19" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.9603569338794616</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.015174876247667</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.9292996824335618</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Virtus Segafredo Bologna</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.9878213802435725</v>
+      </c>
+      <c r="C20" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.9566998244587478</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.050880467418648</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.071703158950359</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Zalgiris Kaunas</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.9810554803788905</v>
+      </c>
+      <c r="C21" t="n">
+        <v>21</v>
+      </c>
+      <c r="D21" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.8191925102399062</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.9883956828694312</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.012869797760321</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>